<commit_message>
v1.72: CC intermediario (reglas ci_pc, sync sin cierre duplicado, migraciones cruces fiat)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/CC_MODELO.xlsx
+++ b/docs/CC_MODELO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucasb/LyP/Pandi/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E07A587F-1B05-044D-A234-874613A5AB8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9879C2AD-11B2-4B44-B8CD-3E05B0D7F962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="3" xr2:uid="{5FE9C384-347E-9A43-BE31-3A982DA54497}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1733" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2257" uniqueCount="264">
   <si>
     <t>Tipo Operacion</t>
   </si>
@@ -517,6 +517,15 @@
     <t>COMBINACION_ID="E,E,E,E" npx playwright test tests/e2e/01-cc-combinaciones.spec.js --reporter=line --workers=1</t>
   </si>
   <si>
+    <t>91-orden-cc.spec.js</t>
+  </si>
+  <si>
+    <t>(smoke 1 orden, sin COMBINACION_ID)</t>
+  </si>
+  <si>
+    <t>npx playwright test tests/e2e/91-orden-cc.spec.js -g "CHEQUE-ARS" --reporter=line --workers=1</t>
+  </si>
+  <si>
     <t>02-cc-tipos-activos-combinaciones.spec.js</t>
   </si>
   <si>
@@ -592,6 +601,12 @@
     <t>TIPO_CODIGO=USD-USD TIPO_USA_INTERMEDIARIO=true COMBINACION_ID="E,E" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
   </si>
   <si>
+    <t>(smoke)</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-usd-usd-int</t>
+  </si>
+  <si>
     <t>USD-ARS + intermediario (inversa)</t>
   </si>
   <si>
@@ -632,6 +647,27 @@
   </si>
   <si>
     <t>TIPO_CODIGO=ARS-USD COMBINACION_ID="E,E" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>(paquete)</t>
+  </si>
+  <si>
+    <t>varios</t>
+  </si>
+  <si>
+    <t>01+02+03</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-activos-completo</t>
+  </si>
+  <si>
+    <t>02+03 sin 01</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-02-03</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-tipos-2tx</t>
   </si>
   <si>
     <r>
@@ -795,12 +831,171 @@
   <si>
     <t>PGPASSWORD='Lmb12044637@' pg_dump -h db.bxwxuzbahewvptarlnxm.supabase.co -p 5432 -U postgres -d postgres --no-owner --no-acl -f ~/Desktop/backup_pandy_$(date +%Y%m%d).sql</t>
   </si>
+  <si>
+    <t>02 completo (todos los tipos 2 tx en un run; incluye EUR si están activos en Supabase)</t>
+  </si>
+  <si>
+    <t>EUR-USD (sin intermediario)</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-eur-usd-sin-int</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-USD COMBINACION_ID="P,P" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-USD COMBINACION_ID="E,P" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-USD COMBINACION_ID="P,E" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-USD COMBINACION_ID="E,E" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>USD-EUR (sin intermediario)</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-usd-eur-sin-int</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=USD-EUR COMBINACION_ID="P,P" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=USD-EUR COMBINACION_ID="E,P" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=USD-EUR COMBINACION_ID="P,E" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=USD-EUR COMBINACION_ID="E,E" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>EUR-ARS (sin intermediario)</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-eur-ars-sin-int</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-ARS COMBINACION_ID="P,P" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-ARS COMBINACION_ID="E,P" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-ARS COMBINACION_ID="P,E" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-ARS COMBINACION_ID="E,E" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>ARS-EUR (sin intermediario)</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-ars-eur-sin-int</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=ARS-EUR COMBINACION_ID="P,P" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=ARS-EUR COMBINACION_ID="E,P" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=ARS-EUR COMBINACION_ID="P,E" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=ARS-EUR COMBINACION_ID="E,E" npx playwright test tests/e2e/02-cc-tipos-activos-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>USD-EUR + intermediario (inversa)</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-usd-eur-int-inversa</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=USD-EUR COMBINACION_ID="P,P" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=USD-EUR COMBINACION_ID="E,P" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=USD-EUR COMBINACION_ID="P,E" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=USD-EUR COMBINACION_ID="E,E" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>EUR-USD + intermediario (inversa)</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-eur-usd-int-inversa</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-USD COMBINACION_ID="P,P" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-USD COMBINACION_ID="E,P" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-USD COMBINACION_ID="P,E" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-USD COMBINACION_ID="E,E" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>EUR-ARS + intermediario (inversa)</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-eur-ars-int-inversa</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-ARS COMBINACION_ID="P,P" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-ARS COMBINACION_ID="E,P" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-ARS COMBINACION_ID="P,E" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=EUR-ARS COMBINACION_ID="E,E" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>ARS-EUR + intermediario (inversa)</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-ars-eur-int-inversa</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=ARS-EUR COMBINACION_ID="P,P" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=ARS-EUR COMBINACION_ID="E,P" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=ARS-EUR COMBINACION_ID="P,E" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>TIPO_CODIGO=ARS-EUR COMBINACION_ID="E,E" npx playwright test tests/e2e/03-cc-intermediario-inversa-combinaciones.spec.js --reporter=line --workers=1</t>
+  </si>
+  <si>
+    <t>Solo EUR sin int (02, 4 tipos)</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-eur-usd-sin-int &amp;&amp; npm run test:e2e-cc-usd-eur-sin-int &amp;&amp; npm run test:e2e-cc-eur-ars-sin-int &amp;&amp; npm run test:e2e-cc-ars-eur-sin-int</t>
+  </si>
+  <si>
+    <t>Solo EUR+int inversa (03, 4 tipos)</t>
+  </si>
+  <si>
+    <t>npm run test:e2e-cc-usd-eur-int-inversa &amp;&amp; npm run test:e2e-cc-eur-usd-int-inversa &amp;&amp; npm run test:e2e-cc-eur-ars-int-inversa &amp;&amp; npm run test:e2e-cc-ars-eur-int-inversa</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1007,6 +1202,19 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Menlo"/>
@@ -1044,7 +1252,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1144,6 +1352,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1269,7 +1483,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="173">
+  <cellXfs count="179">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1627,12 +1841,18 @@
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="34" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="35" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="37" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="36" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="37" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="37" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17952,630 +18172,1190 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D65E1E2-1309-254F-9060-3AB4A003A73C}">
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.33203125" style="169" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="40" style="169" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" style="169" customWidth="1"/>
-    <col min="4" max="4" width="142.1640625" style="169" customWidth="1"/>
-    <col min="5" max="16384" width="10.83203125" style="169"/>
+    <col min="1" max="1" width="29.33203125" style="171" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40" style="171" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" style="171" customWidth="1"/>
+    <col min="4" max="4" width="142.1640625" style="171" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="171"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="168" t="s">
+      <c r="A1" s="170" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="168" t="s">
+      <c r="B1" s="170" t="s">
         <v>138</v>
       </c>
-      <c r="C1" s="168" t="s">
+      <c r="C1" s="170" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="168" t="s">
+      <c r="D1" s="170" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="171" t="s">
+      <c r="A2" s="173" t="s">
         <v>136</v>
       </c>
-      <c r="B2" s="172" t="s">
+      <c r="B2" s="174" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="172" t="s">
+      <c r="C2" s="174" t="s">
         <v>142</v>
       </c>
-      <c r="D2" s="172" t="s">
+      <c r="D2" s="174" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="168" t="s">
+      <c r="A3" s="170" t="s">
         <v>136</v>
       </c>
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="C3" s="170" t="s">
+      <c r="C3" s="172" t="s">
         <v>60</v>
       </c>
-      <c r="D3" s="170" t="s">
+      <c r="D3" s="177" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="168" t="s">
+      <c r="A4" s="170" t="s">
         <v>136</v>
       </c>
-      <c r="B4" s="170" t="s">
+      <c r="B4" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="C4" s="170" t="s">
+      <c r="C4" s="172" t="s">
         <v>66</v>
       </c>
-      <c r="D4" s="170" t="s">
+      <c r="D4" s="177" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="170" t="s">
         <v>136</v>
       </c>
-      <c r="B5" s="170" t="s">
+      <c r="B5" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="C5" s="170" t="s">
+      <c r="C5" s="172" t="s">
         <v>69</v>
       </c>
-      <c r="D5" s="170" t="s">
+      <c r="D5" s="177" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="168" t="s">
+      <c r="A6" s="170" t="s">
         <v>136</v>
       </c>
-      <c r="B6" s="170" t="s">
+      <c r="B6" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="C6" s="170" t="s">
+      <c r="C6" s="172" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="170" t="s">
+      <c r="D6" s="177" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="168" t="s">
+      <c r="A7" s="170" t="s">
         <v>136</v>
       </c>
-      <c r="B7" s="170" t="s">
+      <c r="B7" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="C7" s="170" t="s">
+      <c r="C7" s="172" t="s">
         <v>61</v>
       </c>
-      <c r="D7" s="170" t="s">
+      <c r="D7" s="177" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="168" t="s">
+      <c r="A8" s="170" t="s">
         <v>136</v>
       </c>
-      <c r="B8" s="170" t="s">
+      <c r="B8" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="C8" s="170" t="s">
+      <c r="C8" s="172" t="s">
         <v>73</v>
       </c>
-      <c r="D8" s="170" t="s">
+      <c r="D8" s="177" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="168" t="s">
+      <c r="A9" s="170" t="s">
         <v>136</v>
       </c>
-      <c r="B9" s="170" t="s">
+      <c r="B9" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="C9" s="170" t="s">
+      <c r="C9" s="172" t="s">
         <v>74</v>
       </c>
-      <c r="D9" s="170" t="s">
+      <c r="D9" s="177" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="168" t="s">
+      <c r="A10" s="170" t="s">
         <v>136</v>
       </c>
-      <c r="B10" s="170" t="s">
+      <c r="B10" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="C10" s="170" t="s">
+      <c r="C10" s="172" t="s">
         <v>75</v>
       </c>
-      <c r="D10" s="170" t="s">
+      <c r="D10" s="177" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="168" t="s">
+      <c r="A11" s="170" t="s">
         <v>136</v>
       </c>
-      <c r="B11" s="170" t="s">
+      <c r="B11" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="C11" s="170" t="s">
+      <c r="C11" s="172" t="s">
         <v>62</v>
       </c>
-      <c r="D11" s="170" t="s">
+      <c r="D11" s="177" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="168" t="s">
+      <c r="A12" s="170" t="s">
         <v>136</v>
       </c>
-      <c r="B12" s="170" t="s">
+      <c r="B12" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="C12" s="170" t="s">
+      <c r="C12" s="172" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="170" t="s">
+      <c r="D12" s="177" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="168" t="s">
+      <c r="A13" s="170" t="s">
         <v>136</v>
       </c>
-      <c r="B13" s="170" t="s">
+      <c r="B13" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="C13" s="170" t="s">
+      <c r="C13" s="172" t="s">
         <v>63</v>
       </c>
-      <c r="D13" s="170" t="s">
+      <c r="D13" s="177" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="168" t="s">
+      <c r="A14" s="170" t="s">
         <v>136</v>
       </c>
-      <c r="B14" s="170" t="s">
+      <c r="B14" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="C14" s="170" t="s">
+      <c r="C14" s="172" t="s">
         <v>65</v>
       </c>
-      <c r="D14" s="170" t="s">
+      <c r="D14" s="177" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="171" t="s">
+      <c r="A15" s="173" t="s">
         <v>121</v>
       </c>
-      <c r="B15" s="172" t="s">
-        <v>156</v>
-      </c>
-      <c r="C15" s="172" t="s">
-        <v>157</v>
-      </c>
-      <c r="D15" s="172" t="s">
-        <v>158</v>
+      <c r="B15" s="174" t="s">
+        <v>159</v>
+      </c>
+      <c r="C15" s="174" t="s">
+        <v>160</v>
+      </c>
+      <c r="D15" s="174" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="168" t="s">
+      <c r="A16" s="170" t="s">
         <v>121</v>
       </c>
-      <c r="B16" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C16" s="170" t="s">
+      <c r="B16" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C16" s="172" t="s">
         <v>122</v>
       </c>
-      <c r="D16" s="170" t="s">
+      <c r="D16" s="177" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="170" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17" s="172" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="168" t="s">
+      <c r="C17" s="172" t="s">
+        <v>123</v>
+      </c>
+      <c r="D17" s="177" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="170" t="s">
         <v>121</v>
       </c>
-      <c r="B17" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C17" s="170" t="s">
+      <c r="B18" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C18" s="172" t="s">
+        <v>125</v>
+      </c>
+      <c r="D18" s="177" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="170" t="s">
+        <v>121</v>
+      </c>
+      <c r="B19" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C19" s="172" t="s">
+        <v>127</v>
+      </c>
+      <c r="D19" s="177" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="173" t="s">
+        <v>129</v>
+      </c>
+      <c r="B20" s="174" t="s">
+        <v>159</v>
+      </c>
+      <c r="C20" s="174" t="s">
+        <v>160</v>
+      </c>
+      <c r="D20" s="174" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="170" t="s">
+        <v>129</v>
+      </c>
+      <c r="B21" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C21" s="172" t="s">
+        <v>122</v>
+      </c>
+      <c r="D21" s="177" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="170" t="s">
+        <v>129</v>
+      </c>
+      <c r="B22" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C22" s="172" t="s">
         <v>123</v>
       </c>
-      <c r="D17" s="170" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="168" t="s">
-        <v>121</v>
-      </c>
-      <c r="B18" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C18" s="170" t="s">
+      <c r="D22" s="177" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="170" t="s">
+        <v>129</v>
+      </c>
+      <c r="B23" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C23" s="172" t="s">
         <v>125</v>
       </c>
-      <c r="D18" s="170" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="168" t="s">
-        <v>121</v>
-      </c>
-      <c r="B19" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C19" s="170" t="s">
+      <c r="D23" s="177" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="170" t="s">
+        <v>129</v>
+      </c>
+      <c r="B24" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C24" s="172" t="s">
         <v>127</v>
       </c>
-      <c r="D19" s="170" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="171" t="s">
-        <v>129</v>
-      </c>
-      <c r="B20" s="172" t="s">
-        <v>156</v>
-      </c>
-      <c r="C20" s="172" t="s">
-        <v>157</v>
-      </c>
-      <c r="D20" s="172" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="168" t="s">
-        <v>129</v>
-      </c>
-      <c r="B21" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C21" s="170" t="s">
+      <c r="D24" s="177" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="173" t="s">
+        <v>171</v>
+      </c>
+      <c r="B25" s="174" t="s">
+        <v>159</v>
+      </c>
+      <c r="C25" s="174" t="s">
+        <v>172</v>
+      </c>
+      <c r="D25" s="174" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="170" t="s">
+        <v>171</v>
+      </c>
+      <c r="B26" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C26" s="172" t="s">
         <v>122</v>
       </c>
-      <c r="D21" s="170" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="168" t="s">
-        <v>129</v>
-      </c>
-      <c r="B22" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C22" s="170" t="s">
+      <c r="D26" s="177" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="170" t="s">
+        <v>171</v>
+      </c>
+      <c r="B27" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C27" s="172" t="s">
         <v>123</v>
       </c>
-      <c r="D22" s="170" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="168" t="s">
-        <v>129</v>
-      </c>
-      <c r="B23" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C23" s="170" t="s">
+      <c r="D27" s="177" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" s="170" t="s">
+        <v>171</v>
+      </c>
+      <c r="B28" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C28" s="172" t="s">
         <v>125</v>
       </c>
-      <c r="D23" s="170" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="168" t="s">
-        <v>129</v>
-      </c>
-      <c r="B24" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C24" s="170" t="s">
+      <c r="D28" s="177" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" s="170" t="s">
+        <v>171</v>
+      </c>
+      <c r="B29" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C29" s="172" t="s">
         <v>127</v>
       </c>
-      <c r="D24" s="170" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="171" t="s">
-        <v>168</v>
-      </c>
-      <c r="B25" s="172" t="s">
-        <v>156</v>
-      </c>
-      <c r="C25" s="172" t="s">
-        <v>169</v>
-      </c>
-      <c r="D25" s="172" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="168" t="s">
-        <v>168</v>
-      </c>
-      <c r="B26" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C26" s="170" t="s">
+      <c r="D29" s="177" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" s="173" t="s">
+        <v>178</v>
+      </c>
+      <c r="B30" s="174" t="s">
+        <v>159</v>
+      </c>
+      <c r="C30" s="174" t="s">
+        <v>172</v>
+      </c>
+      <c r="D30" s="174" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="170" t="s">
+        <v>178</v>
+      </c>
+      <c r="B31" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C31" s="172" t="s">
         <v>122</v>
       </c>
-      <c r="D26" s="170" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="168" t="s">
-        <v>168</v>
-      </c>
-      <c r="B27" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C27" s="170" t="s">
+      <c r="D31" s="177" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="170" t="s">
+        <v>178</v>
+      </c>
+      <c r="B32" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C32" s="172" t="s">
         <v>123</v>
       </c>
-      <c r="D27" s="170" t="s">
+      <c r="D32" s="177" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="170" t="s">
+        <v>178</v>
+      </c>
+      <c r="B33" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C33" s="172" t="s">
+        <v>125</v>
+      </c>
+      <c r="D33" s="177" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" s="170" t="s">
+        <v>178</v>
+      </c>
+      <c r="B34" s="172" t="s">
+        <v>159</v>
+      </c>
+      <c r="C34" s="172" t="s">
+        <v>127</v>
+      </c>
+      <c r="D34" s="177" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="173" t="s">
+        <v>186</v>
+      </c>
+      <c r="B35" s="174" t="s">
+        <v>187</v>
+      </c>
+      <c r="C35" s="174" t="s">
+        <v>188</v>
+      </c>
+      <c r="D35" s="174" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" s="170" t="s">
+        <v>186</v>
+      </c>
+      <c r="B36" s="172" t="s">
+        <v>187</v>
+      </c>
+      <c r="C36" s="172" t="s">
+        <v>122</v>
+      </c>
+      <c r="D36" s="177" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" s="170" t="s">
+        <v>186</v>
+      </c>
+      <c r="B37" s="172" t="s">
+        <v>187</v>
+      </c>
+      <c r="C37" s="172" t="s">
+        <v>123</v>
+      </c>
+      <c r="D37" s="177" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" s="170" t="s">
+        <v>186</v>
+      </c>
+      <c r="B38" s="172" t="s">
+        <v>187</v>
+      </c>
+      <c r="C38" s="172" t="s">
+        <v>125</v>
+      </c>
+      <c r="D38" s="177" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="170" t="s">
+        <v>186</v>
+      </c>
+      <c r="B39" s="172" t="s">
+        <v>187</v>
+      </c>
+      <c r="C39" s="172" t="s">
+        <v>127</v>
+      </c>
+      <c r="D39" s="177" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" s="173" t="s">
+        <v>194</v>
+      </c>
+      <c r="B40" s="174" t="s">
+        <v>187</v>
+      </c>
+      <c r="C40" s="174" t="s">
+        <v>188</v>
+      </c>
+      <c r="D40" s="174" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" s="170" t="s">
+        <v>194</v>
+      </c>
+      <c r="B41" s="172" t="s">
+        <v>187</v>
+      </c>
+      <c r="C41" s="172" t="s">
+        <v>122</v>
+      </c>
+      <c r="D41" s="174" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" s="170" t="s">
+        <v>194</v>
+      </c>
+      <c r="B42" s="172" t="s">
+        <v>187</v>
+      </c>
+      <c r="C42" s="172" t="s">
+        <v>123</v>
+      </c>
+      <c r="D42" s="174" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" s="170" t="s">
+        <v>194</v>
+      </c>
+      <c r="B43" s="172" t="s">
+        <v>187</v>
+      </c>
+      <c r="C43" s="172" t="s">
+        <v>125</v>
+      </c>
+      <c r="D43" s="174" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" s="170" t="s">
+        <v>194</v>
+      </c>
+      <c r="B44" s="172" t="s">
+        <v>187</v>
+      </c>
+      <c r="C44" s="172" t="s">
+        <v>127</v>
+      </c>
+      <c r="D44" s="174" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="175" t="s">
+        <v>212</v>
+      </c>
+      <c r="B45" s="176" t="s">
+        <v>159</v>
+      </c>
+      <c r="C45" s="176" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="168" t="s">
-        <v>168</v>
-      </c>
-      <c r="B28" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C28" s="170" t="s">
+      <c r="D45" s="176" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="166" t="s">
+        <v>212</v>
+      </c>
+      <c r="B46" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C46" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D46" s="178" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="166" t="s">
+        <v>212</v>
+      </c>
+      <c r="B47" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C47" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D47" s="178" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="166" t="s">
+        <v>212</v>
+      </c>
+      <c r="B48" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C48" s="167" t="s">
         <v>125</v>
       </c>
-      <c r="D28" s="170" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="168" t="s">
-        <v>168</v>
-      </c>
-      <c r="B29" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C29" s="170" t="s">
+      <c r="D48" s="178" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="166" t="s">
+        <v>212</v>
+      </c>
+      <c r="B49" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C49" s="167" t="s">
         <v>127</v>
       </c>
-      <c r="D29" s="170" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="171" t="s">
-        <v>175</v>
-      </c>
-      <c r="B30" s="172" t="s">
-        <v>156</v>
-      </c>
-      <c r="C30" s="172" t="s">
-        <v>169</v>
-      </c>
-      <c r="D30" s="172" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="168" t="s">
-        <v>175</v>
-      </c>
-      <c r="B31" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C31" s="170" t="s">
+      <c r="D49" s="178" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="175" t="s">
+        <v>218</v>
+      </c>
+      <c r="B50" s="176" t="s">
+        <v>159</v>
+      </c>
+      <c r="C50" s="176" t="s">
+        <v>172</v>
+      </c>
+      <c r="D50" s="176" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="166" t="s">
+        <v>218</v>
+      </c>
+      <c r="B51" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C51" s="167" t="s">
         <v>122</v>
       </c>
-      <c r="D31" s="170" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="168" t="s">
-        <v>175</v>
-      </c>
-      <c r="B32" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C32" s="170" t="s">
+      <c r="D51" s="178" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="166" t="s">
+        <v>218</v>
+      </c>
+      <c r="B52" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C52" s="167" t="s">
         <v>123</v>
       </c>
-      <c r="D32" s="170" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="168" t="s">
-        <v>175</v>
-      </c>
-      <c r="B33" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C33" s="170" t="s">
+      <c r="D52" s="178" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="166" t="s">
+        <v>218</v>
+      </c>
+      <c r="B53" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C53" s="167" t="s">
         <v>125</v>
       </c>
-      <c r="D33" s="170" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="168" t="s">
-        <v>175</v>
-      </c>
-      <c r="B34" s="170" t="s">
-        <v>156</v>
-      </c>
-      <c r="C34" s="170" t="s">
+      <c r="D53" s="178" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="166" t="s">
+        <v>218</v>
+      </c>
+      <c r="B54" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C54" s="167" t="s">
         <v>127</v>
       </c>
-      <c r="D34" s="170" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="171" t="s">
-        <v>181</v>
-      </c>
-      <c r="B35" s="172" t="s">
-        <v>182</v>
-      </c>
-      <c r="C35" s="172" t="s">
-        <v>183</v>
-      </c>
-      <c r="D35" s="172" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="168" t="s">
-        <v>181</v>
-      </c>
-      <c r="B36" s="170" t="s">
-        <v>182</v>
-      </c>
-      <c r="C36" s="170" t="s">
+      <c r="D54" s="178" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="175" t="s">
+        <v>224</v>
+      </c>
+      <c r="B55" s="176" t="s">
+        <v>159</v>
+      </c>
+      <c r="C55" s="176" t="s">
+        <v>172</v>
+      </c>
+      <c r="D55" s="176" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="166" t="s">
+        <v>224</v>
+      </c>
+      <c r="B56" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C56" s="167" t="s">
         <v>122</v>
       </c>
-      <c r="D36" s="170" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="168" t="s">
-        <v>181</v>
-      </c>
-      <c r="B37" s="170" t="s">
-        <v>182</v>
-      </c>
-      <c r="C37" s="170" t="s">
+      <c r="D56" s="178" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="166" t="s">
+        <v>224</v>
+      </c>
+      <c r="B57" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C57" s="167" t="s">
         <v>123</v>
       </c>
-      <c r="D37" s="170" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="168" t="s">
-        <v>181</v>
-      </c>
-      <c r="B38" s="170" t="s">
-        <v>182</v>
-      </c>
-      <c r="C38" s="170" t="s">
+      <c r="D57" s="178" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="166" t="s">
+        <v>224</v>
+      </c>
+      <c r="B58" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C58" s="167" t="s">
         <v>125</v>
       </c>
-      <c r="D38" s="170" t="s">
+      <c r="D58" s="178" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="166" t="s">
+        <v>224</v>
+      </c>
+      <c r="B59" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C59" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D59" s="178" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="175" t="s">
+        <v>230</v>
+      </c>
+      <c r="B60" s="176" t="s">
+        <v>159</v>
+      </c>
+      <c r="C60" s="176" t="s">
+        <v>172</v>
+      </c>
+      <c r="D60" s="176" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="166" t="s">
+        <v>230</v>
+      </c>
+      <c r="B61" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C61" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D61" s="178" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="166" t="s">
+        <v>230</v>
+      </c>
+      <c r="B62" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C62" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D62" s="178" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="166" t="s">
+        <v>230</v>
+      </c>
+      <c r="B63" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C63" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D63" s="178" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="166" t="s">
+        <v>230</v>
+      </c>
+      <c r="B64" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C64" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D64" s="178" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="175" t="s">
+        <v>236</v>
+      </c>
+      <c r="B65" s="176" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="168" t="s">
-        <v>181</v>
-      </c>
-      <c r="B39" s="170" t="s">
-        <v>182</v>
-      </c>
-      <c r="C39" s="170" t="s">
+      <c r="C65" s="176" t="s">
+        <v>188</v>
+      </c>
+      <c r="D65" s="176" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="166" t="s">
+        <v>236</v>
+      </c>
+      <c r="B66" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C66" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D66" s="178" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="166" t="s">
+        <v>236</v>
+      </c>
+      <c r="B67" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C67" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D67" s="178" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="166" t="s">
+        <v>236</v>
+      </c>
+      <c r="B68" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C68" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D68" s="178" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="166" t="s">
+        <v>236</v>
+      </c>
+      <c r="B69" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C69" s="167" t="s">
         <v>127</v>
       </c>
-      <c r="D39" s="170" t="s">
+      <c r="D69" s="178" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="175" t="s">
+        <v>242</v>
+      </c>
+      <c r="B70" s="176" t="s">
+        <v>187</v>
+      </c>
+      <c r="C70" s="176" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="171" t="s">
-        <v>189</v>
-      </c>
-      <c r="B40" s="172" t="s">
-        <v>182</v>
-      </c>
-      <c r="C40" s="172" t="s">
-        <v>183</v>
-      </c>
-      <c r="D40" s="172" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="168" t="s">
-        <v>189</v>
-      </c>
-      <c r="B41" s="170" t="s">
-        <v>182</v>
-      </c>
-      <c r="C41" s="170" t="s">
+      <c r="D70" s="176" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="166" t="s">
+        <v>242</v>
+      </c>
+      <c r="B71" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C71" s="167" t="s">
         <v>122</v>
       </c>
-      <c r="D41" s="170" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="168" t="s">
-        <v>189</v>
-      </c>
-      <c r="B42" s="170" t="s">
-        <v>182</v>
-      </c>
-      <c r="C42" s="170" t="s">
+      <c r="D71" s="177" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="166" t="s">
+        <v>242</v>
+      </c>
+      <c r="B72" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C72" s="167" t="s">
         <v>123</v>
       </c>
-      <c r="D42" s="170" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="168" t="s">
-        <v>189</v>
-      </c>
-      <c r="B43" s="170" t="s">
-        <v>182</v>
-      </c>
-      <c r="C43" s="170" t="s">
+      <c r="D72" s="177" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="166" t="s">
+        <v>242</v>
+      </c>
+      <c r="B73" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C73" s="167" t="s">
         <v>125</v>
       </c>
-      <c r="D43" s="170" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="168" t="s">
-        <v>189</v>
-      </c>
-      <c r="B44" s="170" t="s">
-        <v>182</v>
-      </c>
-      <c r="C44" s="170" t="s">
+      <c r="D73" s="177" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="166" t="s">
+        <v>242</v>
+      </c>
+      <c r="B74" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C74" s="167" t="s">
         <v>127</v>
       </c>
-      <c r="D44" s="170" t="s">
-        <v>194</v>
+      <c r="D74" s="177" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="175" t="s">
+        <v>248</v>
+      </c>
+      <c r="B75" s="176" t="s">
+        <v>187</v>
+      </c>
+      <c r="C75" s="176" t="s">
+        <v>188</v>
+      </c>
+      <c r="D75" s="176" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="166" t="s">
+        <v>248</v>
+      </c>
+      <c r="B76" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C76" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D76" s="178" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="166" t="s">
+        <v>248</v>
+      </c>
+      <c r="B77" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C77" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D77" s="178" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="166" t="s">
+        <v>248</v>
+      </c>
+      <c r="B78" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C78" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D78" s="178" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="166" t="s">
+        <v>248</v>
+      </c>
+      <c r="B79" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C79" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D79" s="178" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="175" t="s">
+        <v>254</v>
+      </c>
+      <c r="B80" s="176" t="s">
+        <v>187</v>
+      </c>
+      <c r="C80" s="176" t="s">
+        <v>188</v>
+      </c>
+      <c r="D80" s="176" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="166" t="s">
+        <v>254</v>
+      </c>
+      <c r="B81" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C81" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D81" s="178" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="166" t="s">
+        <v>254</v>
+      </c>
+      <c r="B82" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C82" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D82" s="178" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="166" t="s">
+        <v>254</v>
+      </c>
+      <c r="B83" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C83" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D83" s="178" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="166" t="s">
+        <v>254</v>
+      </c>
+      <c r="B84" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C84" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D84" s="178" t="s">
+        <v>259</v>
       </c>
     </row>
   </sheetData>
@@ -18585,27 +19365,1296 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DADEDCF5-80F2-CC4F-97BD-F0A0EB15B60F}">
-  <dimension ref="G13:G21"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="146.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="13" spans="7:7" x14ac:dyDescent="0.2">
-      <c r="G13" s="166" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="166" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" s="166" t="s">
+        <v>138</v>
+      </c>
+      <c r="C1" s="166" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1" s="166" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B2" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C2" s="167" t="s">
+        <v>142</v>
+      </c>
+      <c r="D2" s="167" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B3" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" s="167" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="167" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C4" s="167" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" s="167" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C5" s="167" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" s="167" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B6" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C6" s="167" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" s="167" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B7" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C7" s="167" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" s="167" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B8" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C8" s="167" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="167" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B9" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C9" s="167" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" s="167" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B10" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C10" s="167" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="167" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B11" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C11" s="167" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" s="167" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B12" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C12" s="167" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" s="167" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B13" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C13" s="167" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="167" t="s">
+        <v>154</v>
+      </c>
+      <c r="G13" s="168" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B14" s="167" t="s">
+        <v>141</v>
+      </c>
+      <c r="C14" s="167" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="167" t="s">
+        <v>155</v>
+      </c>
+      <c r="G14" s="169" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="166" t="s">
+        <v>136</v>
+      </c>
+      <c r="B15" s="167" t="s">
+        <v>156</v>
+      </c>
+      <c r="C15" s="167" t="s">
+        <v>157</v>
+      </c>
+      <c r="D15" s="167" t="s">
+        <v>158</v>
+      </c>
+      <c r="G15" s="169" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="166" t="s">
+        <v>121</v>
+      </c>
+      <c r="B16" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C16" s="167" t="s">
+        <v>160</v>
+      </c>
+      <c r="D16" s="167" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="166" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C17" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D17" s="167" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="166" t="s">
+        <v>121</v>
+      </c>
+      <c r="B18" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C18" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D18" s="167" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="166" t="s">
+        <v>121</v>
+      </c>
+      <c r="B19" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C19" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D19" s="167" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="166" t="s">
+        <v>121</v>
+      </c>
+      <c r="B20" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C20" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D20" s="167" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="166" t="s">
+        <v>129</v>
+      </c>
+      <c r="B21" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C21" s="167" t="s">
+        <v>160</v>
+      </c>
+      <c r="D21" s="167" t="s">
+        <v>166</v>
+      </c>
+      <c r="G21" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="166" t="s">
+        <v>129</v>
+      </c>
+      <c r="B22" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C22" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D22" s="167" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="166" t="s">
+        <v>129</v>
+      </c>
+      <c r="B23" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C23" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D23" s="167" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="166" t="s">
+        <v>129</v>
+      </c>
+      <c r="B24" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C24" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D24" s="167" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="166" t="s">
+        <v>129</v>
+      </c>
+      <c r="B25" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C25" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D25" s="167" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="166" t="s">
+        <v>171</v>
+      </c>
+      <c r="B26" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C26" s="167" t="s">
+        <v>172</v>
+      </c>
+      <c r="D26" s="167" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="166" t="s">
+        <v>171</v>
+      </c>
+      <c r="B27" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C27" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D27" s="167" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="166" t="s">
+        <v>171</v>
+      </c>
+      <c r="B28" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C28" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D28" s="167" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="166" t="s">
+        <v>171</v>
+      </c>
+      <c r="B29" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C29" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D29" s="167" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="166" t="s">
+        <v>171</v>
+      </c>
+      <c r="B30" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C30" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D30" s="167" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="166" t="s">
+        <v>178</v>
+      </c>
+      <c r="B31" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C31" s="167" t="s">
+        <v>172</v>
+      </c>
+      <c r="D31" s="167" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="166" t="s">
+        <v>178</v>
+      </c>
+      <c r="B32" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C32" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D32" s="167" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="166" t="s">
+        <v>178</v>
+      </c>
+      <c r="B33" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C33" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D33" s="167" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" s="166" t="s">
+        <v>178</v>
+      </c>
+      <c r="B34" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C34" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D34" s="167" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="166" t="s">
+        <v>178</v>
+      </c>
+      <c r="B35" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C35" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D35" s="167" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" s="166" t="s">
+        <v>178</v>
+      </c>
+      <c r="B36" s="167" t="s">
+        <v>156</v>
+      </c>
+      <c r="C36" s="167" t="s">
+        <v>184</v>
+      </c>
+      <c r="D36" s="167" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" s="166" t="s">
+        <v>186</v>
+      </c>
+      <c r="B37" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C37" s="167" t="s">
+        <v>188</v>
+      </c>
+      <c r="D37" s="167" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" s="166" t="s">
+        <v>186</v>
+      </c>
+      <c r="B38" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C38" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D38" s="167" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="166" t="s">
+        <v>186</v>
+      </c>
+      <c r="B39" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C39" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D39" s="167" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" s="166" t="s">
+        <v>186</v>
+      </c>
+      <c r="B40" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C40" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D40" s="167" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" s="166" t="s">
+        <v>186</v>
+      </c>
+      <c r="B41" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C41" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D41" s="167" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" s="166" t="s">
+        <v>194</v>
+      </c>
+      <c r="B42" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C42" s="167" t="s">
+        <v>188</v>
+      </c>
+      <c r="D42" s="167" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" s="166" t="s">
+        <v>194</v>
+      </c>
+      <c r="B43" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C43" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D43" s="167" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" s="166" t="s">
+        <v>194</v>
+      </c>
+      <c r="B44" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C44" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D44" s="167" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="14" spans="7:7" x14ac:dyDescent="0.2">
-      <c r="G14" s="167" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="15" spans="7:7" x14ac:dyDescent="0.2">
-      <c r="G15" s="167" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="21" spans="7:7" x14ac:dyDescent="0.2">
-      <c r="G21" t="s">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" s="166" t="s">
+        <v>194</v>
+      </c>
+      <c r="B45" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C45" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D45" s="167" t="s">
         <v>198</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" s="166" t="s">
+        <v>194</v>
+      </c>
+      <c r="B46" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C46" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D46" s="167" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" s="166" t="s">
+        <v>200</v>
+      </c>
+      <c r="B47" s="167" t="s">
+        <v>201</v>
+      </c>
+      <c r="C47" s="167" t="s">
+        <v>202</v>
+      </c>
+      <c r="D47" s="167" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" s="166" t="s">
+        <v>200</v>
+      </c>
+      <c r="B48" s="167" t="s">
+        <v>201</v>
+      </c>
+      <c r="C48" s="167" t="s">
+        <v>204</v>
+      </c>
+      <c r="D48" s="167" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" s="166" t="s">
+        <v>200</v>
+      </c>
+      <c r="B49" s="167" t="s">
+        <v>201</v>
+      </c>
+      <c r="C49" s="167" t="s">
+        <v>211</v>
+      </c>
+      <c r="D49" s="167" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" s="166" t="s">
+        <v>212</v>
+      </c>
+      <c r="B50" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C50" s="167" t="s">
+        <v>172</v>
+      </c>
+      <c r="D50" s="167" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" s="166" t="s">
+        <v>212</v>
+      </c>
+      <c r="B51" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C51" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D51" s="167" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" s="166" t="s">
+        <v>212</v>
+      </c>
+      <c r="B52" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C52" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D52" s="167" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" s="166" t="s">
+        <v>212</v>
+      </c>
+      <c r="B53" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C53" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D53" s="167" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" s="166" t="s">
+        <v>212</v>
+      </c>
+      <c r="B54" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C54" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D54" s="167" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" s="166" t="s">
+        <v>218</v>
+      </c>
+      <c r="B55" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C55" s="167" t="s">
+        <v>172</v>
+      </c>
+      <c r="D55" s="167" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" s="166" t="s">
+        <v>218</v>
+      </c>
+      <c r="B56" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C56" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D56" s="167" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" s="166" t="s">
+        <v>218</v>
+      </c>
+      <c r="B57" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C57" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D57" s="167" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" s="166" t="s">
+        <v>218</v>
+      </c>
+      <c r="B58" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C58" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D58" s="167" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" s="166" t="s">
+        <v>218</v>
+      </c>
+      <c r="B59" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C59" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D59" s="167" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" s="166" t="s">
+        <v>224</v>
+      </c>
+      <c r="B60" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C60" s="167" t="s">
+        <v>172</v>
+      </c>
+      <c r="D60" s="167" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" s="166" t="s">
+        <v>224</v>
+      </c>
+      <c r="B61" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C61" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D61" s="167" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" s="166" t="s">
+        <v>224</v>
+      </c>
+      <c r="B62" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C62" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D62" s="167" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="166" t="s">
+        <v>224</v>
+      </c>
+      <c r="B63" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C63" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D63" s="167" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="166" t="s">
+        <v>224</v>
+      </c>
+      <c r="B64" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C64" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D64" s="167" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" s="166" t="s">
+        <v>230</v>
+      </c>
+      <c r="B65" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C65" s="167" t="s">
+        <v>172</v>
+      </c>
+      <c r="D65" s="167" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" s="166" t="s">
+        <v>230</v>
+      </c>
+      <c r="B66" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C66" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D66" s="167" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" s="166" t="s">
+        <v>230</v>
+      </c>
+      <c r="B67" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C67" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D67" s="167" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" s="166" t="s">
+        <v>230</v>
+      </c>
+      <c r="B68" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C68" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D68" s="167" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" s="166" t="s">
+        <v>230</v>
+      </c>
+      <c r="B69" s="167" t="s">
+        <v>159</v>
+      </c>
+      <c r="C69" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D69" s="167" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" s="166" t="s">
+        <v>236</v>
+      </c>
+      <c r="B70" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C70" s="167" t="s">
+        <v>188</v>
+      </c>
+      <c r="D70" s="167" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" s="166" t="s">
+        <v>236</v>
+      </c>
+      <c r="B71" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C71" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D71" s="167" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" s="166" t="s">
+        <v>236</v>
+      </c>
+      <c r="B72" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C72" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D72" s="167" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" s="166" t="s">
+        <v>236</v>
+      </c>
+      <c r="B73" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C73" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D73" s="167" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" s="166" t="s">
+        <v>236</v>
+      </c>
+      <c r="B74" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C74" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D74" s="167" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" s="166" t="s">
+        <v>242</v>
+      </c>
+      <c r="B75" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C75" s="167" t="s">
+        <v>188</v>
+      </c>
+      <c r="D75" s="167" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" s="166" t="s">
+        <v>242</v>
+      </c>
+      <c r="B76" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C76" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D76" s="167" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" s="166" t="s">
+        <v>242</v>
+      </c>
+      <c r="B77" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C77" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D77" s="167" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" s="166" t="s">
+        <v>242</v>
+      </c>
+      <c r="B78" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C78" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D78" s="167" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" s="166" t="s">
+        <v>242</v>
+      </c>
+      <c r="B79" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C79" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D79" s="167" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" s="166" t="s">
+        <v>248</v>
+      </c>
+      <c r="B80" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C80" s="167" t="s">
+        <v>188</v>
+      </c>
+      <c r="D80" s="167" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" s="166" t="s">
+        <v>248</v>
+      </c>
+      <c r="B81" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C81" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D81" s="167" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" s="166" t="s">
+        <v>248</v>
+      </c>
+      <c r="B82" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C82" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D82" s="167" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" s="166" t="s">
+        <v>248</v>
+      </c>
+      <c r="B83" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C83" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D83" s="167" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" s="166" t="s">
+        <v>248</v>
+      </c>
+      <c r="B84" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C84" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D84" s="167" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A85" s="166" t="s">
+        <v>254</v>
+      </c>
+      <c r="B85" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C85" s="167" t="s">
+        <v>188</v>
+      </c>
+      <c r="D85" s="167" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A86" s="166" t="s">
+        <v>254</v>
+      </c>
+      <c r="B86" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C86" s="167" t="s">
+        <v>122</v>
+      </c>
+      <c r="D86" s="167" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" s="166" t="s">
+        <v>254</v>
+      </c>
+      <c r="B87" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C87" s="167" t="s">
+        <v>123</v>
+      </c>
+      <c r="D87" s="167" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A88" s="166" t="s">
+        <v>254</v>
+      </c>
+      <c r="B88" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C88" s="167" t="s">
+        <v>125</v>
+      </c>
+      <c r="D88" s="167" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" s="166" t="s">
+        <v>254</v>
+      </c>
+      <c r="B89" s="167" t="s">
+        <v>187</v>
+      </c>
+      <c r="C89" s="167" t="s">
+        <v>127</v>
+      </c>
+      <c r="D89" s="167" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A90" s="166" t="s">
+        <v>200</v>
+      </c>
+      <c r="B90" s="167" t="s">
+        <v>201</v>
+      </c>
+      <c r="C90" s="167" t="s">
+        <v>260</v>
+      </c>
+      <c r="D90" s="167" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A91" s="166" t="s">
+        <v>200</v>
+      </c>
+      <c r="B91" s="167" t="s">
+        <v>201</v>
+      </c>
+      <c r="C91" s="167" t="s">
+        <v>262</v>
+      </c>
+      <c r="D91" s="167" t="s">
+        <v>263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>